<commit_message>
added search function for tool name, type serial, user, status and room
</commit_message>
<xml_diff>
--- a/Planering/scrum.xlsx
+++ b/Planering/scrum.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Yrkesprov_ITUtrustning\Planering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C01195BE-14D8-4B62-9CD0-9C4C2AA79BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A06E9D3-7FAC-4810-95BF-BB789DCD2E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Overview" sheetId="1" r:id="rId1"/>
@@ -264,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -277,11 +277,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -686,7 +698,7 @@
       </c>
       <c r="D2" s="8"/>
       <c r="E2" s="8"/>
-      <c r="F2" s="8">
+      <c r="F2" s="10">
         <v>2</v>
       </c>
     </row>
@@ -699,7 +711,7 @@
       </c>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="7">
+      <c r="F3" s="11">
         <v>1</v>
       </c>
     </row>
@@ -712,7 +724,7 @@
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
-      <c r="F4" s="7">
+      <c r="F4" s="11">
         <v>1</v>
       </c>
       <c r="J4" t="s">
@@ -720,7 +732,7 @@
       </c>
       <c r="K4">
         <f>SUM(F2:F7)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.3">
@@ -732,7 +744,7 @@
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
-      <c r="F5" s="7">
+      <c r="F5" s="11">
         <v>2</v>
       </c>
     </row>
@@ -745,7 +757,9 @@
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
+      <c r="F6" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" spans="2:11" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="7">
@@ -756,7 +770,7 @@
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="F7" s="11"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B8" s="2">
@@ -975,7 +989,9 @@
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
+      <c r="F2" s="12">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="3" spans="1:10" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
@@ -987,7 +1003,7 @@
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
-      <c r="F3" s="10">
+      <c r="F3" s="12">
         <f>SUM(F4:F6)</f>
         <v>0</v>
       </c>
@@ -996,7 +1012,7 @@
       </c>
       <c r="J3" s="9">
         <f>SUM(F10,F7,F3,F2)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -1009,7 +1025,7 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="F4" s="13"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
@@ -1021,7 +1037,7 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="F5" s="14"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
@@ -1033,7 +1049,7 @@
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="F6" s="14"/>
     </row>
     <row r="7" spans="1:10" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="6">
@@ -1045,7 +1061,7 @@
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
-      <c r="F7" s="11">
+      <c r="F7" s="15">
         <f>SUM(F8:F9)</f>
         <v>0</v>
       </c>
@@ -1060,7 +1076,7 @@
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="F8" s="13"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
@@ -1072,7 +1088,7 @@
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="F9" s="14"/>
     </row>
     <row r="10" spans="1:10" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="6">
@@ -1084,7 +1100,7 @@
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
-      <c r="F10" s="11">
+      <c r="F10" s="15">
         <f>SUM(F11:F12)</f>
         <v>0</v>
       </c>
@@ -1099,7 +1115,7 @@
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
+      <c r="F11" s="13"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
@@ -1111,7 +1127,7 @@
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="F12" s="14"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2">

</xml_diff>

<commit_message>
Added a button to allow the user to log out
</commit_message>
<xml_diff>
--- a/Planering/scrum.xlsx
+++ b/Planering/scrum.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Yrkesprov_ITUtrustning\Planering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A06E9D3-7FAC-4810-95BF-BB789DCD2E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20D0C50-95AD-401B-9A5D-00ED470BFB1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1005,14 +1005,14 @@
       <c r="E3" s="5"/>
       <c r="F3" s="12">
         <f>SUM(F4:F6)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="I3" t="s">
         <v>32</v>
       </c>
       <c r="J3" s="9">
         <f>SUM(F10,F7,F3,F2)</f>
-        <v>0.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
@@ -1025,7 +1025,9 @@
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
-      <c r="F4" s="13"/>
+      <c r="F4" s="13">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
@@ -1037,7 +1039,9 @@
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="14"/>
+      <c r="F5" s="14">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
@@ -1063,7 +1067,7 @@
       <c r="E7" s="6"/>
       <c r="F7" s="15">
         <f>SUM(F8:F9)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
@@ -1076,7 +1080,9 @@
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
-      <c r="F8" s="13"/>
+      <c r="F8" s="13">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
@@ -1102,7 +1108,7 @@
       <c r="E10" s="6"/>
       <c r="F10" s="15">
         <f>SUM(F11:F12)</f>
-        <v>0</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -1115,7 +1121,9 @@
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
-      <c r="F11" s="13"/>
+      <c r="F11" s="13">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
@@ -1127,7 +1135,9 @@
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
-      <c r="F12" s="14"/>
+      <c r="F12" s="14">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2">

</xml_diff>